<commit_message>
finish scraping from 2023,1,1
</commit_message>
<xml_diff>
--- a/database_package/table_schema.xlsx
+++ b/database_package/table_schema.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\marcus\workplace\Github\finance_project\database_package\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C99919D-2CAC-4F7C-A7FB-05D79BC19CBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC2CF6CB-3AB6-4A70-9F8C-443B74A98C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t>column</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -79,11 +79,19 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>INTEGER</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>FLOAT(4)</t>
+  </si>
+  <si>
+    <t>Capital Gains</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FLOAT(4)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VARCHAR(10)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -417,7 +425,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" customWidth="1"/>
@@ -445,7 +453,7 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
@@ -453,7 +461,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
@@ -461,7 +469,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
@@ -469,7 +477,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
@@ -485,7 +493,7 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -493,15 +501,23 @@
         <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>13</v>
+      <c r="B11" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
scraping finance statement ,Unable to upload to database(because column name)
</commit_message>
<xml_diff>
--- a/database_package/table_schema.xlsx
+++ b/database_package/table_schema.xlsx
@@ -1,96 +1,239 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\marcus\workplace\Github\finance_project\database_package\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC2CF6CB-3AB6-4A70-9F8C-443B74A98C4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202920E6-C8A9-4414-8607-76F60D20B640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="stock_price" sheetId="1" r:id="rId1"/>
+    <sheet name="finance_statement" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="71">
   <si>
     <t>column</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>data_type</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Date</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>DATE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Open</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FLOAT(4)</t>
   </si>
   <si>
     <t>High</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Low</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Close</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Volume</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>BIGINT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Dividends</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Stock Splits</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Capital Gains</t>
   </si>
   <si>
     <t>stock_id</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>FLOAT(4)</t>
-  </si>
-  <si>
-    <t>Capital Gains</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>FLOAT(4)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>VARCHAR(10)</t>
+  </si>
+  <si>
+    <t>Tax Effect Of Unusual Items</t>
+  </si>
+  <si>
+    <t>FLOAT(16)</t>
+  </si>
+  <si>
+    <t>Tax Rate For Calcs</t>
+  </si>
+  <si>
+    <t>Normalized EBITDA</t>
+  </si>
+  <si>
+    <t>Total Unusual Items</t>
+  </si>
+  <si>
+    <t>Total Unusual Items Excluding Goodwill</t>
+  </si>
+  <si>
+    <t>Net Income From Continuing Operation Net Minority Interest</t>
+  </si>
+  <si>
+    <t>Reconciled Depreciation</t>
+  </si>
+  <si>
+    <t>Reconciled Cost Of Revenue</t>
+  </si>
+  <si>
+    <t>EBITDA</t>
+  </si>
+  <si>
+    <t>EBIT</t>
+  </si>
+  <si>
+    <t>Net Interest Income</t>
+  </si>
+  <si>
+    <t>Interest Expense</t>
+  </si>
+  <si>
+    <t>Interest Income</t>
+  </si>
+  <si>
+    <t>Normalized Income</t>
+  </si>
+  <si>
+    <t>Net Income From Continuing And Discontinued Operation</t>
+  </si>
+  <si>
+    <t>Total Expenses</t>
+  </si>
+  <si>
+    <t>Total Operating Income As Reported</t>
+  </si>
+  <si>
+    <t>Diluted Average Shares</t>
+  </si>
+  <si>
+    <t>Basic Average Shares</t>
+  </si>
+  <si>
+    <t>Diluted EPS</t>
+  </si>
+  <si>
+    <t>Basic EPS</t>
+  </si>
+  <si>
+    <t>Diluted NI Availto Com Stockholders</t>
+  </si>
+  <si>
+    <t>Net Income Common Stockholders</t>
+  </si>
+  <si>
+    <t>Net Income</t>
+  </si>
+  <si>
+    <t>Minority Interests</t>
+  </si>
+  <si>
+    <t>Net Income Including Noncontrolling Interests</t>
+  </si>
+  <si>
+    <t>Net Income Continuous Operations</t>
+  </si>
+  <si>
+    <t>Tax Provision</t>
+  </si>
+  <si>
+    <t>Pretax Income</t>
+  </si>
+  <si>
+    <t>Other Income Expense</t>
+  </si>
+  <si>
+    <t>Other Non Operating Income Expenses</t>
+  </si>
+  <si>
+    <t>Special Income Charges</t>
+  </si>
+  <si>
+    <t>Gain On Sale Of Business</t>
+  </si>
+  <si>
+    <t>Write Off</t>
+  </si>
+  <si>
+    <t>Earnings From Equity Interest</t>
+  </si>
+  <si>
+    <t>Gain On Sale Of Security</t>
+  </si>
+  <si>
+    <t>Net Non Operating Interest Income Expense</t>
+  </si>
+  <si>
+    <t>Total Other Finance Cost</t>
+  </si>
+  <si>
+    <t>Interest Expense Non Operating</t>
+  </si>
+  <si>
+    <t>Interest Income Non Operating</t>
+  </si>
+  <si>
+    <t>Operating Income</t>
+  </si>
+  <si>
+    <t>Operating Expense</t>
+  </si>
+  <si>
+    <t>Other Operating Expenses</t>
+  </si>
+  <si>
+    <t>Research And Development</t>
+  </si>
+  <si>
+    <t>Selling General And Administration</t>
+  </si>
+  <si>
+    <t>Selling And Marketing Expense</t>
+  </si>
+  <si>
+    <t>General And Administrative Expense</t>
+  </si>
+  <si>
+    <t>Other Gand A</t>
+  </si>
+  <si>
+    <t>Gross Profit</t>
+  </si>
+  <si>
+    <t>Cost Of Revenue</t>
+  </si>
+  <si>
+    <t>Total Revenue</t>
+  </si>
+  <si>
+    <t>Operating Revenue</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Otherunder Preferred Stock Dividend</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -98,7 +241,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -121,6 +264,13 @@
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="新細明體"/>
+      <family val="1"/>
+      <charset val="136"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -130,7 +280,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -138,13 +288,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -448,80 +616,543 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B10" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B11" s="1" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:B56"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="57.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>34</v>
+      </c>
+      <c r="B19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>45</v>
+      </c>
+      <c r="B30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>46</v>
+      </c>
+      <c r="B31" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>47</v>
+      </c>
+      <c r="B32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>48</v>
+      </c>
+      <c r="B33" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>49</v>
+      </c>
+      <c r="B34" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>50</v>
+      </c>
+      <c r="B35" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>51</v>
+      </c>
+      <c r="B36" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>53</v>
+      </c>
+      <c r="B38" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>57</v>
+      </c>
+      <c r="B42" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>58</v>
+      </c>
+      <c r="B43" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>59</v>
+      </c>
+      <c r="B44" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>60</v>
+      </c>
+      <c r="B45" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>61</v>
+      </c>
+      <c r="B46" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>64</v>
+      </c>
+      <c r="B49" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>65</v>
+      </c>
+      <c r="B50" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>66</v>
+      </c>
+      <c r="B51" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>67</v>
+      </c>
+      <c r="B52" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>68</v>
+      </c>
+      <c r="B53" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>70</v>
+      </c>
+      <c r="B54" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>69</v>
+      </c>
+      <c r="B55" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>14</v>
+      </c>
+      <c r="B56" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
basic information has been done
</commit_message>
<xml_diff>
--- a/database_package/table_schema.xlsx
+++ b/database_package/table_schema.xlsx
@@ -1,27 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\marcus\workplace\Github\finance_project\database_package\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D33278-E243-4E95-B649-D51FFDA668F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76D514A-F80C-4BEC-934C-2FDBF43BD303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="stock_price" sheetId="1" r:id="rId1"/>
     <sheet name="finance_statement" sheetId="2" r:id="rId2"/>
+    <sheet name="basic_information" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="38">
   <si>
     <t>column</t>
   </si>
@@ -84,6 +85,75 @@
   </si>
   <si>
     <t>stock_id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>股票代號</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>股票名稱</t>
+  </si>
+  <si>
+    <t>產業別</t>
+  </si>
+  <si>
+    <t>上市/上櫃</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>上市日期</t>
+  </si>
+  <si>
+    <t>上櫃日期</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>資本額</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>每股面值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>目前市值</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>公司債發行</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>發行股數</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>特別股</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>盈餘分派頻率</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>董事長</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VARCHAR(20)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VARCHAR(4)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VARCHAR(8)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VARCHAR(100)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -612,4 +682,139 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46234476-975F-41B1-9A44-E614D8DD1C8E}">
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>